<commit_message>
Update forecasts and add manual tracker
</commit_message>
<xml_diff>
--- a/Manual Tracker/Forecast History.xlsx
+++ b/Manual Tracker/Forecast History.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://friedkingroup-my.sharepoint.com/personal/mconner_gsfsgroup_com/Documents/Documents/Github/Weather/Manual Tracker/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="54" documentId="11_F25DC773A252ABDACC104895015A47085ADE58F1" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BEFF8E5F-F38D-4955-88F0-E817FF5216DF}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -18,12 +24,151 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="42">
+  <si>
+    <t>station_id</t>
+  </si>
+  <si>
+    <t>name</t>
+  </si>
+  <si>
+    <t>lat</t>
+  </si>
+  <si>
+    <t>lon</t>
+  </si>
+  <si>
+    <t>timezone</t>
+  </si>
+  <si>
+    <t>KHOU</t>
+  </si>
+  <si>
+    <t>Houston Hobby</t>
+  </si>
+  <si>
+    <t>America/Chicago</t>
+  </si>
+  <si>
+    <t>KNYC</t>
+  </si>
+  <si>
+    <t>New York Central Park</t>
+  </si>
+  <si>
+    <t>America/New_York</t>
+  </si>
+  <si>
+    <t>KDFW</t>
+  </si>
+  <si>
+    <t>Dallas Fort Worth</t>
+  </si>
+  <si>
+    <t>KMIA</t>
+  </si>
+  <si>
+    <t>Miami International</t>
+  </si>
+  <si>
+    <t>KBOS</t>
+  </si>
+  <si>
+    <t>Boston Logan</t>
+  </si>
+  <si>
+    <t>KSEA</t>
+  </si>
+  <si>
+    <t>Seattle Tacoma</t>
+  </si>
+  <si>
+    <t>America/Los_Angeles</t>
+  </si>
+  <si>
+    <t>KLAX</t>
+  </si>
+  <si>
+    <t>LA International</t>
+  </si>
+  <si>
+    <t>forecast site</t>
+  </si>
+  <si>
+    <t>https://forecast.weather.gov/MapClick.php?lat=33.9435233&amp;lon=-118.4085523</t>
+  </si>
+  <si>
+    <t>https://forecast.weather.gov/MapClick.php?lat=29.6524&amp;lon=-95.2772</t>
+  </si>
+  <si>
+    <t>https://forecast.weather.gov/MapClick.php?lat=40.713&amp;lon=-74.0072</t>
+  </si>
+  <si>
+    <t>https://forecast.weather.gov/MapClick.php?lat=32.8975&amp;lon=-97.0444</t>
+  </si>
+  <si>
+    <t>https://forecast.weather.gov/MapClick.php?lat=25.795&amp;lon=-80.2798</t>
+  </si>
+  <si>
+    <t>https://forecast.weather.gov/MapClick.php?lat=42.3635&amp;lon=-71.0181</t>
+  </si>
+  <si>
+    <t>https://forecast.weather.gov/MapClick.php?lat=47.4436&amp;lon=-122.3029</t>
+  </si>
+  <si>
+    <t>KMDW</t>
+  </si>
+  <si>
+    <t>Chicago Midway</t>
+  </si>
+  <si>
+    <t>https://forecast.weather.gov/MapClick.php?lat=41.7885&amp;lon=-87.7417</t>
+  </si>
+  <si>
+    <t>KAUS</t>
+  </si>
+  <si>
+    <t>Austin Bergstrom</t>
+  </si>
+  <si>
+    <t>https://forecast.weather.gov/MapClick.php?lat=30.1945&amp;lon=-97.6699</t>
+  </si>
+  <si>
+    <t>KSFO</t>
+  </si>
+  <si>
+    <t>San Francisco International</t>
+  </si>
+  <si>
+    <t>https://forecast.weather.gov/MapClick.php?lat=37.6188&amp;lon=-122.3758</t>
+  </si>
+  <si>
+    <t>KOKC</t>
+  </si>
+  <si>
+    <t>OKC Will Rogers</t>
+  </si>
+  <si>
+    <t>https://forecast.weather.gov/MapClick.php?lat=35.4456&amp;lon=-97.6019</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -46,13 +191,16 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -330,10 +478,271 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:F12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="20.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2">
+        <v>29.645399999999999</v>
+      </c>
+      <c r="D2">
+        <v>-95.278899999999993</v>
+      </c>
+      <c r="E2" t="s">
+        <v>7</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3">
+        <v>40.713000000000001</v>
+      </c>
+      <c r="D3">
+        <v>-74.007199999999997</v>
+      </c>
+      <c r="E3" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C4">
+        <v>32.897500000000001</v>
+      </c>
+      <c r="D4">
+        <v>-97.044399999999996</v>
+      </c>
+      <c r="E4" t="s">
+        <v>7</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>13</v>
+      </c>
+      <c r="B5" t="s">
+        <v>14</v>
+      </c>
+      <c r="C5">
+        <v>25.795000000000002</v>
+      </c>
+      <c r="D5">
+        <v>-80.279799999999994</v>
+      </c>
+      <c r="E5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>15</v>
+      </c>
+      <c r="B6" t="s">
+        <v>16</v>
+      </c>
+      <c r="C6">
+        <v>42.363500000000002</v>
+      </c>
+      <c r="D6">
+        <v>-71.018100000000004</v>
+      </c>
+      <c r="E6" t="s">
+        <v>10</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>17</v>
+      </c>
+      <c r="B7" t="s">
+        <v>18</v>
+      </c>
+      <c r="C7">
+        <v>47.443600000000004</v>
+      </c>
+      <c r="D7">
+        <v>-122.30289999999999</v>
+      </c>
+      <c r="E7" t="s">
+        <v>19</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>20</v>
+      </c>
+      <c r="B8" t="s">
+        <v>21</v>
+      </c>
+      <c r="C8">
+        <v>33.943523300000003</v>
+      </c>
+      <c r="D8">
+        <v>-118.4085523</v>
+      </c>
+      <c r="E8" t="s">
+        <v>19</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>30</v>
+      </c>
+      <c r="B9" t="s">
+        <v>31</v>
+      </c>
+      <c r="C9">
+        <v>41.788499999999999</v>
+      </c>
+      <c r="D9">
+        <v>-87.741699999999994</v>
+      </c>
+      <c r="E9" t="s">
+        <v>7</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>33</v>
+      </c>
+      <c r="B10" t="s">
+        <v>34</v>
+      </c>
+      <c r="C10">
+        <v>30.194500000000001</v>
+      </c>
+      <c r="D10">
+        <v>-97.669899999999998</v>
+      </c>
+      <c r="E10" t="s">
+        <v>7</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>36</v>
+      </c>
+      <c r="B11" t="s">
+        <v>37</v>
+      </c>
+      <c r="C11">
+        <v>37.6188</v>
+      </c>
+      <c r="D11">
+        <v>-122.3758</v>
+      </c>
+      <c r="E11" t="s">
+        <v>19</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>39</v>
+      </c>
+      <c r="B12" t="s">
+        <v>40</v>
+      </c>
+      <c r="C12">
+        <v>35.445599999999999</v>
+      </c>
+      <c r="D12">
+        <v>-97.601900000000001</v>
+      </c>
+      <c r="E12" t="s">
+        <v>7</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>41</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="F10" r:id="rId1" xr:uid="{61360C6E-CA7A-4D70-82D8-81EA68937D71}"/>
+    <hyperlink ref="F11" r:id="rId2" xr:uid="{8D33D9D2-28CA-4AD2-8714-E08045AEDD60}"/>
+    <hyperlink ref="F12" r:id="rId3" xr:uid="{2F2AD209-0774-4306-9039-25F6585123C3}"/>
+    <hyperlink ref="F2" r:id="rId4" xr:uid="{208E681D-E255-42FF-85B2-A0B785D112AF}"/>
+    <hyperlink ref="F3" r:id="rId5" xr:uid="{1C45D61C-5C5D-402F-8046-7C3B6FD41487}"/>
+    <hyperlink ref="F4" r:id="rId6" xr:uid="{D0E0FA00-AAEC-48E1-B72A-C4298C71DF1E}"/>
+    <hyperlink ref="F5" r:id="rId7" xr:uid="{18B0C74C-77CA-4F4B-9362-B64A1D9717F2}"/>
+    <hyperlink ref="F6" r:id="rId8" xr:uid="{C6B7E366-C33B-46D4-B10F-67B5388760E6}"/>
+    <hyperlink ref="F7" r:id="rId9" xr:uid="{C4987F40-3385-4732-8B98-E010CBF59DDC}"/>
+    <hyperlink ref="F8" r:id="rId10" xr:uid="{1F5947BA-9CFC-4E02-9288-AD5DB11556A7}"/>
+    <hyperlink ref="F9" r:id="rId11" xr:uid="{C8C98A14-AE8A-4D96-A129-A4B9720458FE}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>